<commit_message>
Update Readme and plot
</commit_message>
<xml_diff>
--- a/Sources_and_Python_Code/Data/Gym_Locations_RAW_FILE.xlsx
+++ b/Sources_and_Python_Code/Data/Gym_Locations_RAW_FILE.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universityofexeteruk-my.sharepoint.com/personal/sf584_exeter_ac_uk/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Local_Work_HardDrive\Data Science\Empirical project\Sources_and_Python_Code\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A067D829-FB98-4B68-916D-FAFB4EFF7198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6AF6D16E-8FFE-42EE-93CC-72F4CC2118D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="970" windowWidth="19060" windowHeight="8470" xr2:uid="{CAB61DA6-1AFF-4491-935F-32198C383519}"/>
+    <workbookView xWindow="140" yWindow="270" windowWidth="19060" windowHeight="8470" xr2:uid="{CAB61DA6-1AFF-4491-935F-32198C383519}"/>
   </bookViews>
   <sheets>
     <sheet name="gym_locations" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="199">
   <si>
     <t>name</t>
   </si>
@@ -52,9 +52,6 @@
     <t>post_olympics</t>
   </si>
   <si>
-    <t>era</t>
-  </si>
-  <si>
     <t>The Castle Climbing Centre</t>
   </si>
   <si>
@@ -67,9 +64,6 @@
     <t>https://castle-climbing.co.uk</t>
   </si>
   <si>
-    <t>1990s</t>
-  </si>
-  <si>
     <t>Mile End Climbing Wall</t>
   </si>
   <si>
@@ -88,21 +82,12 @@
     <t>https://www.awesomewalls.co.uk</t>
   </si>
   <si>
-    <t>2000s</t>
-  </si>
-  <si>
-    <t>The Warehouse Climbing Centre Gloucester</t>
-  </si>
-  <si>
     <t>Gloucester</t>
   </si>
   <si>
     <t>South West</t>
   </si>
   <si>
-    <t>https://www.warehouse-climbing.com</t>
-  </si>
-  <si>
     <t>Alien Rock</t>
   </si>
   <si>
@@ -127,9 +112,6 @@
     <t>Glasgow climbing centre</t>
   </si>
   <si>
-    <t>Glascow</t>
-  </si>
-  <si>
     <t>https://glasgowclimbingcentre.com/</t>
   </si>
   <si>
@@ -154,27 +136,18 @@
     <t>West Midlands</t>
   </si>
   <si>
-    <t>https://redpointclimbing.co.uk</t>
-  </si>
-  <si>
     <t>Quay Climbing Centre</t>
   </si>
   <si>
     <t>Exeter</t>
   </si>
   <si>
-    <t>https://quayclimbing.com</t>
-  </si>
-  <si>
     <t>Wolverhampton Climbing Centre</t>
   </si>
   <si>
     <t>Wolverhampton</t>
   </si>
   <si>
-    <t>https://www.wolverhamptonclimbing.co.uk</t>
-  </si>
-  <si>
     <t>The Boardroom Climbing Centre</t>
   </si>
   <si>
@@ -193,9 +166,6 @@
     <t>Wales</t>
   </si>
   <si>
-    <t>https://www.bouldersclimbing.com</t>
-  </si>
-  <si>
     <t>The Arch Climbing Wall</t>
   </si>
   <si>
@@ -217,21 +187,12 @@
     <t>North East</t>
   </si>
   <si>
-    <t>https://sunderlandwall.co.uk</t>
-  </si>
-  <si>
     <t>ROKT Climbing Gym</t>
   </si>
   <si>
     <t>Brighouse</t>
   </si>
   <si>
-    <t>https://www.rokt.co.uk</t>
-  </si>
-  <si>
-    <t>2010s</t>
-  </si>
-  <si>
     <t>Rock City Climbing Centre</t>
   </si>
   <si>
@@ -277,27 +238,18 @@
     <t>The Climbing Hangar Liverpool</t>
   </si>
   <si>
-    <t>https://www.theclimbinghangar.com</t>
-  </si>
-  <si>
     <t>Chimera Climbing &amp; Fitness</t>
   </si>
   <si>
     <t>Southampton</t>
   </si>
   <si>
-    <t>https://chimeraclimbing.co.uk</t>
-  </si>
-  <si>
     <t>Big Rock Climbing Centre</t>
   </si>
   <si>
     <t>Milton Keynes</t>
   </si>
   <si>
-    <t>https://bigrockclimbingcentre.co.uk</t>
-  </si>
-  <si>
     <t>Beacon Climbing Centre</t>
   </si>
   <si>
@@ -328,54 +280,30 @@
     <t>Vauxwall</t>
   </si>
   <si>
-    <t>https://vauxwall.com</t>
-  </si>
-  <si>
     <t>The Climbing Lab</t>
   </si>
   <si>
     <t>https://www.climbinglab.co.uk</t>
   </si>
   <si>
-    <t>Vertical Limits Nottingham</t>
-  </si>
-  <si>
-    <t>Nottingham</t>
-  </si>
-  <si>
     <t>East Midlands</t>
   </si>
   <si>
-    <t>https://www.verticallimitsclimbing.co.uk</t>
-  </si>
-  <si>
     <t>Depot Climbing Birmingham</t>
   </si>
   <si>
-    <t>https://depotclimbing.com</t>
-  </si>
-  <si>
     <t>The Climbing Station</t>
   </si>
   <si>
     <t>Loughborough</t>
   </si>
   <si>
-    <t>https://theclimbingstation.co.uk</t>
-  </si>
-  <si>
     <t>The Climbing Hangar Swansea</t>
   </si>
   <si>
     <t>Swansea</t>
   </si>
   <si>
-    <t>Boulder Central</t>
-  </si>
-  <si>
-    <t>https://bouldercentral.co.uk</t>
-  </si>
-  <si>
     <t>Rainbow Rocket Colchester</t>
   </si>
   <si>
@@ -385,9 +313,6 @@
     <t>East</t>
   </si>
   <si>
-    <t>https://www.rainbowrocket.co.uk</t>
-  </si>
-  <si>
     <t>Awesome Walls Stockport</t>
   </si>
   <si>
@@ -409,9 +334,6 @@
     <t>Harrogate</t>
   </si>
   <si>
-    <t>https://harrowall.com</t>
-  </si>
-  <si>
     <t>The Climbing Hangar Plymouth</t>
   </si>
   <si>
@@ -424,9 +346,6 @@
     <t>Ellesmere Port</t>
   </si>
   <si>
-    <t>https://www.theclimbinghut.com</t>
-  </si>
-  <si>
     <t>TCA The Prop Store</t>
   </si>
   <si>
@@ -436,51 +355,27 @@
     <t>https://theclimbingacademy.com</t>
   </si>
   <si>
-    <t>Rock UK Summit Centre</t>
-  </si>
-  <si>
-    <t>Trelewis</t>
-  </si>
-  <si>
-    <t>https://rockuk.org/centres/summit-centre/</t>
-  </si>
-  <si>
     <t>Parthian Climbing Manchester</t>
   </si>
   <si>
     <t>https://parthianclimbing.com</t>
   </si>
   <si>
-    <t>The Climbing Academy Newcastle</t>
-  </si>
-  <si>
     <t>Newcastle</t>
   </si>
   <si>
     <t>BlocHaus Climbing</t>
   </si>
   <si>
-    <t>Norwich</t>
-  </si>
-  <si>
-    <t>https://www.blochaus.co.uk</t>
-  </si>
-  <si>
     <t>Clip N Climb Cambridge</t>
   </si>
   <si>
     <t>Cambridge</t>
   </si>
   <si>
-    <t>https://cambridge.clipnclimb.com</t>
-  </si>
-  <si>
     <t>Flashpoint Bristol</t>
   </si>
   <si>
-    <t>https://flashpointbristol.co.uk</t>
-  </si>
-  <si>
     <t>Volume 1 Climbing</t>
   </si>
   <si>
@@ -517,15 +412,9 @@
     <t>https://www.prestonwall.co.uk</t>
   </si>
   <si>
-    <t>2020s</t>
-  </si>
-  <si>
     <t>Rock Over Sheffield</t>
   </si>
   <si>
-    <t>Depot Climbing Newcastle</t>
-  </si>
-  <si>
     <t>City Bouldering Aldgate</t>
   </si>
   <si>
@@ -535,18 +424,6 @@
     <t>Rock Up Birmingham</t>
   </si>
   <si>
-    <t>https://www.rockup.co.uk</t>
-  </si>
-  <si>
-    <t>Stronghold Bouldering</t>
-  </si>
-  <si>
-    <t>Reading</t>
-  </si>
-  <si>
-    <t>Industry report</t>
-  </si>
-  <si>
     <t>Flashpoint Swindon</t>
   </si>
   <si>
@@ -568,9 +445,6 @@
     <t>Climb Newcastle The Pool</t>
   </si>
   <si>
-    <t>https://climbnewcastle.co.uk</t>
-  </si>
-  <si>
     <t>Rise Climbing</t>
   </si>
   <si>
@@ -583,12 +457,6 @@
     <t>LCC EustonWall</t>
   </si>
   <si>
-    <t>https://londonclimbingcentres.co.uk</t>
-  </si>
-  <si>
-    <t>Bloc Climbing</t>
-  </si>
-  <si>
     <t>Indirock</t>
   </si>
   <si>
@@ -616,9 +484,6 @@
     <t>Big Depot Leeds</t>
   </si>
   <si>
-    <t>https://www.depotclimbing.co.uk</t>
-  </si>
-  <si>
     <t>Rhino Boulder</t>
   </si>
   <si>
@@ -637,14 +502,128 @@
     <t>Scarborough</t>
   </si>
   <si>
-    <t>https://cavca.org.uk</t>
+    <t>https://climbingdistrict.uk/climbing-gym/london-fields/</t>
+  </si>
+  <si>
+    <t>Stronghold Climbing</t>
+  </si>
+  <si>
+    <t>https://www.blochausclimbing.com/</t>
+  </si>
+  <si>
+    <t>https://www.rise-climbing.com/</t>
+  </si>
+  <si>
+    <t>Deeside</t>
+  </si>
+  <si>
+    <t>https://www.270climbing.com/</t>
+  </si>
+  <si>
+    <t>270 climbing</t>
+  </si>
+  <si>
+    <t>https://www.redpointbirmingham.co.uk/</t>
+  </si>
+  <si>
+    <t>https://quayclimbingcentre.co.uk/</t>
+  </si>
+  <si>
+    <t>https://www.wolfmountainactivitycentre.co.uk/</t>
+  </si>
+  <si>
+    <t>https://bouldersuk.com/</t>
+  </si>
+  <si>
+    <t>https://redpointbristol.co.uk/</t>
+  </si>
+  <si>
+    <t>https://sunderlandwall.com/</t>
+  </si>
+  <si>
+    <t>https://www.rokt.co.uk/</t>
+  </si>
+  <si>
+    <t>https://www.theclimbinghangar.com/locations/liverpool-north</t>
+  </si>
+  <si>
+    <t>https://www.chimeraclimbing.com/</t>
+  </si>
+  <si>
+    <t>Canterbury</t>
+  </si>
+  <si>
+    <t>https://www.bigrockclimbing.com/</t>
+  </si>
+  <si>
+    <t>https://londonclimbingcentres.co.uk/centre/vauxwest/</t>
+  </si>
+  <si>
+    <t>https://www.depotclimbing.co.uk/birmingham/</t>
+  </si>
+  <si>
+    <t>https://theclimbingstation.com/</t>
+  </si>
+  <si>
+    <t>https://www.theclimbinghangar.com/locations/swansea</t>
+  </si>
+  <si>
+    <t>Boulder Shack</t>
+  </si>
+  <si>
+    <t>https://bouldershack.co.uk/</t>
+  </si>
+  <si>
+    <t>https://rainbowrocket.cc/</t>
+  </si>
+  <si>
+    <t>https://www.awesomewalls.co.uk/stockport/</t>
+  </si>
+  <si>
+    <t>https://www.depotclimbing.co.uk/big-depot/</t>
+  </si>
+  <si>
+    <t>https://londonclimbingcentres.co.uk/centre/harrowall/</t>
+  </si>
+  <si>
+    <t>https://www.theclimbinghangar.com/locations/plymouth</t>
+  </si>
+  <si>
+    <t>https://www.climbinghut.com/</t>
+  </si>
+  <si>
+    <t>https://www.theclimbingacademy.com/locations/the-prop-store/</t>
+  </si>
+  <si>
+    <t>https://www.clipnclimbcambridge.co.uk/</t>
+  </si>
+  <si>
+    <t>https://flashpointbristol.com/</t>
+  </si>
+  <si>
+    <t>https://www.rock-up.co.uk/locations/birmingham</t>
+  </si>
+  <si>
+    <t>https://www.climbnewcastle.com/</t>
+  </si>
+  <si>
+    <t>https://londonclimbingcentres.co.uk/centre/eustonwall/</t>
+  </si>
+  <si>
+    <t>https://www.depotclimbing.co.uk/manchester/?_gl=1%2Aq9klp8%2A_up%2AMQ..%2A_ga%2ANTg0MzYxNDYzLjE3NzgyMjYzMjk.%2A_ga_7TXZCZ3B9X%2AczE3NzgyMjYzMjgkbzEkZzAkdDE3NzgyMjYzMjgkajYwJGwwJGgw%2A_ga_XKDQRJ4PB4%2AczE3NzgyMjYzMjgkbzEkZzAkdDE3NzgyMjYzMjgkajYwJGwwJGg3NTkzODk3MjM.</t>
+  </si>
+  <si>
+    <t>https://www.depotclimbing.co.uk/big-depot-manchester/</t>
+  </si>
+  <si>
+    <t>https://cavca.org.uk/street-rocks/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -775,6 +754,14 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1077,7 +1064,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -1120,12 +1107,14 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -1159,6 +1148,7 @@
     <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
     <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Hyperlink" xfId="42" builtinId="8"/>
     <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
     <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
@@ -1499,10 +1489,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6989338E-88CD-4709-AED2-065BB2C0AC0C}">
-  <dimension ref="A1:K76"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="8" max="8" width="11.36328125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1533,168 +1526,153 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" t="s">
-        <v>12</v>
-      </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D2">
         <v>1995</v>
       </c>
       <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
         <v>14</v>
       </c>
-      <c r="G2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H2" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I2" t="b">
-        <v>1</v>
-      </c>
-      <c r="J2" t="b">
-        <v>0</v>
-      </c>
-      <c r="K2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>16</v>
-      </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D3">
         <v>1995</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
         <v>17</v>
       </c>
-      <c r="G3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I3" t="b">
-        <v>1</v>
-      </c>
-      <c r="J3" t="b">
-        <v>0</v>
-      </c>
-      <c r="K3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+      <c r="C4" t="s">
         <v>18</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>20</v>
       </c>
       <c r="D4">
         <v>2003</v>
       </c>
       <c r="E4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>166</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
         <v>21</v>
       </c>
-      <c r="G4" t="b">
-        <v>1</v>
-      </c>
-      <c r="H4" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I4" t="b">
-        <v>1</v>
-      </c>
-      <c r="J4" t="b">
-        <v>0</v>
-      </c>
-      <c r="K4" t="s">
+      <c r="D5">
+        <v>2024</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="B6" t="s">
         <v>23</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C6" t="s">
         <v>24</v>
-      </c>
-      <c r="C5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5">
-        <v>2005</v>
-      </c>
-      <c r="E5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" t="s">
-        <v>26</v>
-      </c>
-      <c r="G5" t="b">
-        <v>1</v>
-      </c>
-      <c r="H5" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I5" t="b">
-        <v>1</v>
-      </c>
-      <c r="J5" t="b">
-        <v>0</v>
-      </c>
-      <c r="K5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" t="s">
-        <v>29</v>
       </c>
       <c r="D6">
         <v>2005</v>
       </c>
       <c r="E6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" t="s">
-        <v>30</v>
+        <v>12</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>25</v>
       </c>
       <c r="G6" t="b">
         <v>1</v>
@@ -1708,98 +1686,89 @@
       <c r="J6" t="b">
         <v>0</v>
       </c>
-      <c r="K6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7">
+        <v>2018</v>
+      </c>
+      <c r="E7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C7" t="s">
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>29</v>
       </c>
-      <c r="D7">
-        <v>2005</v>
-      </c>
-      <c r="E7" t="s">
-        <v>32</v>
-      </c>
-      <c r="F7" t="s">
-        <v>33</v>
-      </c>
-      <c r="G7" t="b">
-        <v>1</v>
-      </c>
-      <c r="H7" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I7" t="b">
-        <v>1</v>
-      </c>
-      <c r="J7" t="b">
-        <v>0</v>
-      </c>
-      <c r="K7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>34</v>
-      </c>
       <c r="B8" t="s">
-        <v>35</v>
+        <v>109</v>
       </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D8">
         <v>2005</v>
       </c>
       <c r="E8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I8" t="b">
+        <v>1</v>
+      </c>
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s">
         <v>32</v>
       </c>
-      <c r="F8" t="s">
-        <v>36</v>
-      </c>
-      <c r="G8" t="b">
-        <v>1</v>
-      </c>
-      <c r="H8" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I8" t="b">
-        <v>1</v>
-      </c>
-      <c r="J8" t="b">
-        <v>0</v>
-      </c>
-      <c r="K8" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B9" t="s">
-        <v>38</v>
-      </c>
       <c r="C9" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D9">
         <v>2006</v>
       </c>
       <c r="E9" t="s">
-        <v>32</v>
-      </c>
-      <c r="F9" t="s">
-        <v>40</v>
+        <v>27</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="G9" t="b">
         <v>1</v>
@@ -1813,28 +1782,25 @@
       <c r="J9" t="b">
         <v>0</v>
       </c>
-      <c r="K9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C10" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="D10">
         <v>2006</v>
       </c>
       <c r="E10" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" t="s">
-        <v>44</v>
+        <v>12</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>167</v>
       </c>
       <c r="G10" t="b">
         <v>1</v>
@@ -1848,98 +1814,89 @@
       <c r="J10" t="b">
         <v>0</v>
       </c>
-      <c r="K10" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="B11" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D11">
         <v>2008</v>
       </c>
       <c r="E11" t="s">
-        <v>13</v>
-      </c>
-      <c r="F11" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I11" t="b">
+        <v>1</v>
+      </c>
+      <c r="J11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12">
+        <v>2009</v>
+      </c>
+      <c r="E12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I12" t="b">
+        <v>1</v>
+      </c>
+      <c r="J12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" t="s">
+        <v>164</v>
+      </c>
+      <c r="C13" t="s">
         <v>47</v>
-      </c>
-      <c r="G11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H11" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I11" t="b">
-        <v>1</v>
-      </c>
-      <c r="J11" t="b">
-        <v>0</v>
-      </c>
-      <c r="K11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>48</v>
-      </c>
-      <c r="B12" t="s">
-        <v>49</v>
-      </c>
-      <c r="C12" t="s">
-        <v>43</v>
-      </c>
-      <c r="D12">
-        <v>2008</v>
-      </c>
-      <c r="E12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" t="s">
-        <v>50</v>
-      </c>
-      <c r="G12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H12" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I12" t="b">
-        <v>1</v>
-      </c>
-      <c r="J12" t="b">
-        <v>0</v>
-      </c>
-      <c r="K12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>51</v>
-      </c>
-      <c r="B13" t="s">
-        <v>52</v>
-      </c>
-      <c r="C13" t="s">
-        <v>39</v>
       </c>
       <c r="D13">
         <v>2009</v>
       </c>
       <c r="E13" t="s">
-        <v>32</v>
-      </c>
-      <c r="F13" t="s">
-        <v>53</v>
+        <v>27</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>44</v>
       </c>
       <c r="G13" t="b">
         <v>1</v>
@@ -1953,28 +1910,25 @@
       <c r="J13" t="b">
         <v>0</v>
       </c>
-      <c r="K13" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="B14" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="C14" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="D14">
         <v>2009</v>
       </c>
       <c r="E14" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" t="s">
-        <v>57</v>
+        <v>12</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>170</v>
       </c>
       <c r="G14" t="b">
         <v>1</v>
@@ -1988,28 +1942,25 @@
       <c r="J14" t="b">
         <v>0</v>
       </c>
-      <c r="K14" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="B15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D15">
         <v>2010</v>
       </c>
       <c r="E15" t="s">
-        <v>32</v>
-      </c>
-      <c r="F15" t="s">
-        <v>59</v>
+        <v>27</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>49</v>
       </c>
       <c r="G15" t="b">
         <v>1</v>
@@ -2023,28 +1974,25 @@
       <c r="J15" t="b">
         <v>0</v>
       </c>
-      <c r="K15" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="B16" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="C16" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D16">
         <v>2010</v>
       </c>
       <c r="E16" t="s">
-        <v>13</v>
-      </c>
-      <c r="F16" t="s">
-        <v>44</v>
+        <v>12</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>171</v>
       </c>
       <c r="G16" t="b">
         <v>1</v>
@@ -2058,28 +2006,25 @@
       <c r="J16" t="b">
         <v>0</v>
       </c>
-      <c r="K16" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="B17" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="C17" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="D17">
         <v>2010</v>
       </c>
       <c r="E17" t="s">
-        <v>13</v>
-      </c>
-      <c r="F17" t="s">
-        <v>65</v>
+        <v>12</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>172</v>
       </c>
       <c r="G17" t="b">
         <v>1</v>
@@ -2093,28 +2038,25 @@
       <c r="J17" t="b">
         <v>0</v>
       </c>
-      <c r="K17" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="B18" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="C18" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D18">
         <v>2011</v>
       </c>
       <c r="E18" t="s">
-        <v>13</v>
-      </c>
-      <c r="F18" t="s">
-        <v>68</v>
+        <v>12</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>173</v>
       </c>
       <c r="G18" t="b">
         <v>1</v>
@@ -2128,28 +2070,25 @@
       <c r="J18" t="b">
         <v>0</v>
       </c>
-      <c r="K18" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="B19" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="C19" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D19">
         <v>2011</v>
       </c>
       <c r="E19" t="s">
-        <v>13</v>
-      </c>
-      <c r="F19" t="s">
-        <v>72</v>
+        <v>12</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>59</v>
       </c>
       <c r="G19" t="b">
         <v>1</v>
@@ -2163,28 +2102,25 @@
       <c r="J19" t="b">
         <v>0</v>
       </c>
-      <c r="K19" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="B20" t="s">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="C20" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="D20">
         <v>2012</v>
       </c>
       <c r="E20" t="s">
-        <v>32</v>
-      </c>
-      <c r="F20" t="s">
-        <v>76</v>
+        <v>27</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>63</v>
       </c>
       <c r="G20" t="b">
         <v>1</v>
@@ -2198,28 +2134,25 @@
       <c r="J20" t="b">
         <v>0</v>
       </c>
-      <c r="K20" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="B21" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C21" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D21">
         <v>2012</v>
       </c>
       <c r="E21" t="s">
-        <v>13</v>
-      </c>
-      <c r="F21" t="s">
-        <v>78</v>
+        <v>12</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="G21" t="b">
         <v>1</v>
@@ -2233,63 +2166,57 @@
       <c r="J21" t="b">
         <v>0</v>
       </c>
-      <c r="K21" t="s">
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>66</v>
+      </c>
+      <c r="B22" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" t="s">
+        <v>33</v>
+      </c>
+      <c r="D22">
+        <v>1991</v>
+      </c>
+      <c r="E22" t="s">
+        <v>12</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G22" t="b">
+        <v>1</v>
+      </c>
+      <c r="H22" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I22" t="b">
+        <v>1</v>
+      </c>
+      <c r="J22" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>68</v>
+      </c>
+      <c r="B23" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>79</v>
-      </c>
-      <c r="B22" t="s">
-        <v>38</v>
-      </c>
-      <c r="C22" t="s">
-        <v>39</v>
-      </c>
-      <c r="D22">
-        <v>2012</v>
-      </c>
-      <c r="E22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F22" t="s">
-        <v>80</v>
-      </c>
-      <c r="G22" t="b">
-        <v>1</v>
-      </c>
-      <c r="H22" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I22" t="b">
-        <v>1</v>
-      </c>
-      <c r="J22" t="b">
-        <v>0</v>
-      </c>
-      <c r="K22" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>81</v>
-      </c>
-      <c r="B23" t="s">
-        <v>82</v>
-      </c>
       <c r="C23" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="D23">
         <v>2013</v>
       </c>
       <c r="E23" t="s">
-        <v>13</v>
-      </c>
-      <c r="F23" t="s">
-        <v>83</v>
+        <v>12</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>70</v>
       </c>
       <c r="G23" t="b">
         <v>1</v>
@@ -2303,28 +2230,25 @@
       <c r="J23" t="b">
         <v>0</v>
       </c>
-      <c r="K23" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="B24" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C24" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D24">
         <v>2014</v>
       </c>
       <c r="E24" t="s">
-        <v>32</v>
-      </c>
-      <c r="F24" t="s">
-        <v>85</v>
+        <v>27</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>174</v>
       </c>
       <c r="G24" t="b">
         <v>1</v>
@@ -2338,28 +2262,25 @@
       <c r="J24" t="b">
         <v>0</v>
       </c>
-      <c r="K24" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="B25" t="s">
-        <v>87</v>
+        <v>176</v>
       </c>
       <c r="C25" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="D25">
         <v>2014</v>
       </c>
       <c r="E25" t="s">
-        <v>13</v>
-      </c>
-      <c r="F25" t="s">
-        <v>88</v>
+        <v>12</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>175</v>
       </c>
       <c r="G25" t="b">
         <v>1</v>
@@ -2373,28 +2294,25 @@
       <c r="J25" t="b">
         <v>0</v>
       </c>
-      <c r="K25" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="B26" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="C26" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="D26">
         <v>2014</v>
       </c>
       <c r="E26" t="s">
-        <v>13</v>
-      </c>
-      <c r="F26" t="s">
-        <v>91</v>
+        <v>12</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>177</v>
       </c>
       <c r="G26" t="b">
         <v>1</v>
@@ -2408,28 +2326,25 @@
       <c r="J26" t="b">
         <v>0</v>
       </c>
-      <c r="K26" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="B27" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="C27" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="D27">
         <v>2014</v>
       </c>
       <c r="E27" t="s">
-        <v>13</v>
-      </c>
-      <c r="F27" t="s">
-        <v>94</v>
+        <v>12</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>78</v>
       </c>
       <c r="G27" t="b">
         <v>1</v>
@@ -2443,28 +2358,25 @@
       <c r="J27" t="b">
         <v>0</v>
       </c>
-      <c r="K27" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="B28" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="C28" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D28">
-        <v>2014</v>
+        <v>2013</v>
       </c>
       <c r="E28" t="s">
-        <v>32</v>
-      </c>
-      <c r="F28" t="s">
-        <v>97</v>
+        <v>27</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>81</v>
       </c>
       <c r="G28" t="b">
         <v>1</v>
@@ -2478,28 +2390,25 @@
       <c r="J28" t="b">
         <v>0</v>
       </c>
-      <c r="K28" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="B29" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="C29" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D29">
         <v>2015</v>
       </c>
       <c r="E29" t="s">
-        <v>32</v>
-      </c>
-      <c r="F29" t="s">
-        <v>100</v>
+        <v>27</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="G29" t="b">
         <v>1</v>
@@ -2513,28 +2422,25 @@
       <c r="J29" t="b">
         <v>0</v>
       </c>
-      <c r="K29" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>101</v>
+        <v>85</v>
       </c>
       <c r="B30" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C30" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D30">
         <v>2015</v>
       </c>
       <c r="E30" t="s">
-        <v>32</v>
-      </c>
-      <c r="F30" t="s">
-        <v>102</v>
+        <v>27</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>178</v>
       </c>
       <c r="G30" t="b">
         <v>1</v>
@@ -2548,28 +2454,25 @@
       <c r="J30" t="b">
         <v>0</v>
       </c>
-      <c r="K30" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>103</v>
+        <v>86</v>
       </c>
       <c r="B31" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="C31" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D31">
         <v>2015</v>
       </c>
       <c r="E31" t="s">
-        <v>32</v>
-      </c>
-      <c r="F31" t="s">
-        <v>104</v>
+        <v>27</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>87</v>
       </c>
       <c r="G31" t="b">
         <v>1</v>
@@ -2583,28 +2486,25 @@
       <c r="J31" t="b">
         <v>0</v>
       </c>
-      <c r="K31" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>105</v>
+        <v>89</v>
       </c>
       <c r="B32" t="s">
-        <v>106</v>
+        <v>36</v>
       </c>
       <c r="C32" t="s">
-        <v>107</v>
+        <v>37</v>
       </c>
       <c r="D32">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="E32" t="s">
-        <v>13</v>
-      </c>
-      <c r="F32" t="s">
-        <v>108</v>
+        <v>27</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>179</v>
       </c>
       <c r="G32" t="b">
         <v>1</v>
@@ -2618,28 +2518,25 @@
       <c r="J32" t="b">
         <v>0</v>
       </c>
-      <c r="K32" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="B33" t="s">
-        <v>42</v>
+        <v>91</v>
       </c>
       <c r="C33" t="s">
-        <v>43</v>
+        <v>88</v>
       </c>
       <c r="D33">
         <v>2016</v>
       </c>
       <c r="E33" t="s">
-        <v>32</v>
-      </c>
-      <c r="F33" t="s">
-        <v>110</v>
+        <v>27</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>180</v>
       </c>
       <c r="G33" t="b">
         <v>1</v>
@@ -2653,28 +2550,25 @@
       <c r="J33" t="b">
         <v>0</v>
       </c>
-      <c r="K33" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>111</v>
+        <v>92</v>
       </c>
       <c r="B34" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="C34" t="s">
-        <v>107</v>
+        <v>47</v>
       </c>
       <c r="D34">
         <v>2016</v>
       </c>
       <c r="E34" t="s">
-        <v>32</v>
-      </c>
-      <c r="F34" t="s">
-        <v>113</v>
+        <v>27</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>181</v>
       </c>
       <c r="G34" t="b">
         <v>1</v>
@@ -2688,28 +2582,25 @@
       <c r="J34" t="b">
         <v>0</v>
       </c>
-      <c r="K34" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>114</v>
+        <v>182</v>
       </c>
       <c r="B35" t="s">
-        <v>115</v>
+        <v>73</v>
       </c>
       <c r="C35" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="D35">
         <v>2016</v>
       </c>
       <c r="E35" t="s">
-        <v>32</v>
-      </c>
-      <c r="F35" t="s">
-        <v>85</v>
+        <v>27</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>183</v>
       </c>
       <c r="G35" t="b">
         <v>1</v>
@@ -2723,28 +2614,25 @@
       <c r="J35" t="b">
         <v>0</v>
       </c>
-      <c r="K35" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>116</v>
+        <v>94</v>
       </c>
       <c r="B36" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="C36" t="s">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="D36">
         <v>2017</v>
       </c>
       <c r="E36" t="s">
-        <v>32</v>
-      </c>
-      <c r="F36" t="s">
-        <v>117</v>
+        <v>12</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>184</v>
       </c>
       <c r="G36" t="b">
         <v>1</v>
@@ -2758,28 +2646,25 @@
       <c r="J36" t="b">
         <v>0</v>
       </c>
-      <c r="K36" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>118</v>
+        <v>97</v>
       </c>
       <c r="B37" t="s">
-        <v>119</v>
+        <v>98</v>
       </c>
       <c r="C37" t="s">
-        <v>120</v>
+        <v>18</v>
       </c>
       <c r="D37">
         <v>2017</v>
       </c>
       <c r="E37" t="s">
-        <v>13</v>
-      </c>
-      <c r="F37" t="s">
-        <v>121</v>
+        <v>12</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>185</v>
       </c>
       <c r="G37" t="b">
         <v>1</v>
@@ -2793,28 +2678,25 @@
       <c r="J37" t="b">
         <v>0</v>
       </c>
-      <c r="K37" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>122</v>
+        <v>99</v>
       </c>
       <c r="B38" t="s">
-        <v>123</v>
+        <v>11</v>
       </c>
       <c r="C38" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D38">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="E38" t="s">
-        <v>13</v>
-      </c>
-      <c r="F38" t="s">
-        <v>21</v>
+        <v>27</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>100</v>
       </c>
       <c r="G38" t="b">
         <v>1</v>
@@ -2828,28 +2710,25 @@
       <c r="J38" t="b">
         <v>0</v>
       </c>
-      <c r="K38" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>124</v>
+        <v>101</v>
       </c>
       <c r="B39" t="s">
-        <v>12</v>
+        <v>43</v>
       </c>
       <c r="C39" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="D39">
         <v>2018</v>
       </c>
       <c r="E39" t="s">
-        <v>32</v>
-      </c>
-      <c r="F39" t="s">
-        <v>125</v>
+        <v>27</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>186</v>
       </c>
       <c r="G39" t="b">
         <v>1</v>
@@ -2863,28 +2742,25 @@
       <c r="J39" t="b">
         <v>0</v>
       </c>
-      <c r="K39" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>126</v>
+        <v>102</v>
       </c>
       <c r="B40" t="s">
-        <v>52</v>
+        <v>103</v>
       </c>
       <c r="C40" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D40">
         <v>2018</v>
       </c>
       <c r="E40" t="s">
-        <v>32</v>
-      </c>
-      <c r="F40" t="s">
-        <v>110</v>
+        <v>27</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>187</v>
       </c>
       <c r="G40" t="b">
         <v>1</v>
@@ -2898,28 +2774,25 @@
       <c r="J40" t="b">
         <v>0</v>
       </c>
-      <c r="K40" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>127</v>
+        <v>104</v>
       </c>
       <c r="B41" t="s">
-        <v>128</v>
+        <v>105</v>
       </c>
       <c r="C41" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="D41">
         <v>2018</v>
       </c>
       <c r="E41" t="s">
-        <v>32</v>
-      </c>
-      <c r="F41" t="s">
-        <v>129</v>
+        <v>27</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>188</v>
       </c>
       <c r="G41" t="b">
         <v>1</v>
@@ -2933,28 +2806,25 @@
       <c r="J41" t="b">
         <v>0</v>
       </c>
-      <c r="K41" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>130</v>
+        <v>106</v>
       </c>
       <c r="B42" t="s">
-        <v>131</v>
+        <v>107</v>
       </c>
       <c r="C42" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="D42">
         <v>2018</v>
       </c>
       <c r="E42" t="s">
-        <v>32</v>
-      </c>
-      <c r="F42" t="s">
-        <v>85</v>
+        <v>27</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>189</v>
       </c>
       <c r="G42" t="b">
         <v>1</v>
@@ -2968,28 +2838,25 @@
       <c r="J42" t="b">
         <v>0</v>
       </c>
-      <c r="K42" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>132</v>
+        <v>108</v>
       </c>
       <c r="B43" t="s">
-        <v>133</v>
+        <v>109</v>
       </c>
       <c r="C43" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D43">
         <v>2018</v>
       </c>
       <c r="E43" t="s">
-        <v>32</v>
-      </c>
-      <c r="F43" t="s">
-        <v>134</v>
+        <v>27</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>190</v>
       </c>
       <c r="G43" t="b">
         <v>1</v>
@@ -3003,28 +2870,25 @@
       <c r="J43" t="b">
         <v>0</v>
       </c>
-      <c r="K43" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>135</v>
+        <v>111</v>
       </c>
       <c r="B44" t="s">
-        <v>136</v>
+        <v>83</v>
       </c>
       <c r="C44" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="D44">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="E44" t="s">
-        <v>32</v>
-      </c>
-      <c r="F44" t="s">
-        <v>137</v>
+        <v>27</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>112</v>
       </c>
       <c r="G44" t="b">
         <v>1</v>
@@ -3038,28 +2902,25 @@
       <c r="J44" t="b">
         <v>0</v>
       </c>
-      <c r="K44" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>138</v>
+        <v>115</v>
       </c>
       <c r="B45" t="s">
-        <v>139</v>
+        <v>116</v>
       </c>
       <c r="C45" t="s">
-        <v>56</v>
+        <v>96</v>
       </c>
       <c r="D45">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="E45" t="s">
-        <v>13</v>
-      </c>
-      <c r="F45" t="s">
-        <v>140</v>
+        <v>12</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>191</v>
       </c>
       <c r="G45" t="b">
         <v>1</v>
@@ -3073,28 +2934,25 @@
       <c r="J45" t="b">
         <v>0</v>
       </c>
-      <c r="K45" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>141</v>
+        <v>117</v>
       </c>
       <c r="B46" t="s">
-        <v>99</v>
+        <v>51</v>
       </c>
       <c r="C46" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D46">
         <v>2019</v>
       </c>
       <c r="E46" t="s">
-        <v>32</v>
-      </c>
-      <c r="F46" t="s">
-        <v>142</v>
+        <v>27</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>192</v>
       </c>
       <c r="G46" t="b">
         <v>1</v>
@@ -3108,28 +2966,25 @@
       <c r="J46" t="b">
         <v>0</v>
       </c>
-      <c r="K46" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>143</v>
+        <v>118</v>
       </c>
       <c r="B47" t="s">
-        <v>144</v>
+        <v>119</v>
       </c>
       <c r="C47" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D47">
         <v>2019</v>
       </c>
       <c r="E47" t="s">
-        <v>13</v>
-      </c>
-      <c r="F47" t="s">
-        <v>137</v>
+        <v>27</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>120</v>
       </c>
       <c r="G47" t="b">
         <v>1</v>
@@ -3143,168 +2998,153 @@
       <c r="J47" t="b">
         <v>0</v>
       </c>
-      <c r="K47" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>145</v>
+        <v>121</v>
       </c>
       <c r="B48" t="s">
-        <v>146</v>
+        <v>51</v>
       </c>
       <c r="C48" t="s">
-        <v>120</v>
+        <v>21</v>
       </c>
       <c r="D48">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="E48" t="s">
+        <v>27</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="G48" t="b">
+        <v>1</v>
+      </c>
+      <c r="H48" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I48" t="b">
+        <v>0</v>
+      </c>
+      <c r="J48" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>122</v>
+      </c>
+      <c r="B49" t="s">
+        <v>11</v>
+      </c>
+      <c r="C49" t="s">
+        <v>11</v>
+      </c>
+      <c r="D49">
+        <v>2020</v>
+      </c>
+      <c r="E49" t="s">
+        <v>27</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="G49" t="b">
+        <v>1</v>
+      </c>
+      <c r="H49" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I49" t="b">
+        <v>0</v>
+      </c>
+      <c r="J49" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>124</v>
+      </c>
+      <c r="B50" t="s">
+        <v>125</v>
+      </c>
+      <c r="C50" t="s">
+        <v>33</v>
+      </c>
+      <c r="D50">
+        <v>2020</v>
+      </c>
+      <c r="E50" t="s">
+        <v>12</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G50" t="b">
+        <v>1</v>
+      </c>
+      <c r="H50" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I50" t="b">
+        <v>0</v>
+      </c>
+      <c r="J50" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>127</v>
+      </c>
+      <c r="B51" t="s">
+        <v>128</v>
+      </c>
+      <c r="C51" t="s">
+        <v>18</v>
+      </c>
+      <c r="D51">
+        <v>2021</v>
+      </c>
+      <c r="E51" t="s">
+        <v>12</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="G51" t="b">
+        <v>1</v>
+      </c>
+      <c r="H51" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I51" t="b">
+        <v>0</v>
+      </c>
+      <c r="J51" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>130</v>
+      </c>
+      <c r="B52" t="s">
         <v>32</v>
       </c>
-      <c r="F48" t="s">
-        <v>147</v>
-      </c>
-      <c r="G48" t="b">
-        <v>1</v>
-      </c>
-      <c r="H48" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I48" t="b">
-        <v>1</v>
-      </c>
-      <c r="J48" t="b">
-        <v>0</v>
-      </c>
-      <c r="K48" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
-        <v>148</v>
-      </c>
-      <c r="B49" t="s">
-        <v>149</v>
-      </c>
-      <c r="C49" t="s">
-        <v>120</v>
-      </c>
-      <c r="D49">
-        <v>2019</v>
-      </c>
-      <c r="E49" t="s">
-        <v>13</v>
-      </c>
-      <c r="F49" t="s">
-        <v>150</v>
-      </c>
-      <c r="G49" t="b">
-        <v>1</v>
-      </c>
-      <c r="H49" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I49" t="b">
-        <v>1</v>
-      </c>
-      <c r="J49" t="b">
-        <v>0</v>
-      </c>
-      <c r="K49" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
-        <v>151</v>
-      </c>
-      <c r="B50" t="s">
-        <v>61</v>
-      </c>
-      <c r="C50" t="s">
-        <v>25</v>
-      </c>
-      <c r="D50">
-        <v>2019</v>
-      </c>
-      <c r="E50" t="s">
-        <v>32</v>
-      </c>
-      <c r="F50" t="s">
-        <v>152</v>
-      </c>
-      <c r="G50" t="b">
-        <v>1</v>
-      </c>
-      <c r="H50" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I50" t="b">
-        <v>1</v>
-      </c>
-      <c r="J50" t="b">
-        <v>0</v>
-      </c>
-      <c r="K50" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
-        <v>153</v>
-      </c>
-      <c r="B51" t="s">
-        <v>154</v>
-      </c>
-      <c r="C51" t="s">
-        <v>75</v>
-      </c>
-      <c r="D51">
-        <v>2019</v>
-      </c>
-      <c r="E51" t="s">
-        <v>32</v>
-      </c>
-      <c r="F51" t="s">
-        <v>155</v>
-      </c>
-      <c r="G51" t="b">
-        <v>1</v>
-      </c>
-      <c r="H51" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I51" t="b">
-        <v>1</v>
-      </c>
-      <c r="J51" t="b">
-        <v>0</v>
-      </c>
-      <c r="K51" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
-        <v>156</v>
-      </c>
-      <c r="B52" t="s">
-        <v>61</v>
-      </c>
       <c r="C52" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="D52">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E52" t="s">
-        <v>32</v>
-      </c>
-      <c r="F52" t="s">
-        <v>137</v>
+        <v>27</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>84</v>
       </c>
       <c r="G52" t="b">
         <v>1</v>
@@ -3316,30 +3156,27 @@
         <v>0</v>
       </c>
       <c r="J52" t="b">
-        <v>0</v>
-      </c>
-      <c r="K52" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>157</v>
+        <v>131</v>
       </c>
       <c r="B53" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C53" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D53">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E53" t="s">
-        <v>32</v>
-      </c>
-      <c r="F53" t="s">
-        <v>158</v>
+        <v>27</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>132</v>
       </c>
       <c r="G53" t="b">
         <v>1</v>
@@ -3351,65 +3188,59 @@
         <v>0</v>
       </c>
       <c r="J53" t="b">
-        <v>0</v>
-      </c>
-      <c r="K53" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>159</v>
+        <v>133</v>
       </c>
       <c r="B54" t="s">
-        <v>160</v>
+        <v>36</v>
       </c>
       <c r="C54" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D54">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E54" t="s">
-        <v>13</v>
-      </c>
-      <c r="F54" t="s">
+        <v>27</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="G54" t="b">
+        <v>1</v>
+      </c>
+      <c r="H54" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I54" t="b">
+        <v>0</v>
+      </c>
+      <c r="J54" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
         <v>161</v>
       </c>
-      <c r="G54" t="b">
-        <v>1</v>
-      </c>
-      <c r="H54" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I54" t="b">
-        <v>0</v>
-      </c>
-      <c r="J54" t="b">
-        <v>0</v>
-      </c>
-      <c r="K54" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
-        <v>162</v>
-      </c>
       <c r="B55" t="s">
-        <v>163</v>
+        <v>11</v>
       </c>
       <c r="C55" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D55">
         <v>2021</v>
       </c>
       <c r="E55" t="s">
-        <v>13</v>
-      </c>
-      <c r="F55" t="s">
-        <v>164</v>
+        <v>27</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>160</v>
       </c>
       <c r="G55" t="b">
         <v>1</v>
@@ -3423,28 +3254,25 @@
       <c r="J55" t="b">
         <v>1</v>
       </c>
-      <c r="K55" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>166</v>
+        <v>134</v>
       </c>
       <c r="B56" t="s">
-        <v>38</v>
+        <v>135</v>
       </c>
       <c r="C56" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="D56">
         <v>2021</v>
       </c>
       <c r="E56" t="s">
-        <v>32</v>
-      </c>
-      <c r="F56" t="s">
-        <v>100</v>
+        <v>27</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>136</v>
       </c>
       <c r="G56" t="b">
         <v>1</v>
@@ -3458,28 +3286,25 @@
       <c r="J56" t="b">
         <v>1</v>
       </c>
-      <c r="K56" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>167</v>
+        <v>137</v>
       </c>
       <c r="B57" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C57" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D57">
         <v>2021</v>
       </c>
       <c r="E57" t="s">
-        <v>32</v>
-      </c>
-      <c r="F57" t="s">
-        <v>110</v>
+        <v>12</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>139</v>
       </c>
       <c r="G57" t="b">
         <v>1</v>
@@ -3493,28 +3318,25 @@
       <c r="J57" t="b">
         <v>1</v>
       </c>
-      <c r="K57" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>168</v>
+        <v>140</v>
       </c>
       <c r="B58" t="s">
-        <v>12</v>
+        <v>113</v>
       </c>
       <c r="C58" t="s">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="D58">
         <v>2021</v>
       </c>
       <c r="E58" t="s">
-        <v>32</v>
-      </c>
-      <c r="F58" t="s">
-        <v>169</v>
+        <v>27</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>194</v>
       </c>
       <c r="G58" t="b">
         <v>1</v>
@@ -3528,28 +3350,25 @@
       <c r="J58" t="b">
         <v>1</v>
       </c>
-      <c r="K58" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>170</v>
+        <v>141</v>
       </c>
       <c r="B59" t="s">
-        <v>42</v>
+        <v>11</v>
       </c>
       <c r="C59" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="D59">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="E59" t="s">
-        <v>32</v>
-      </c>
-      <c r="F59" t="s">
-        <v>171</v>
+        <v>27</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>163</v>
       </c>
       <c r="G59" t="b">
         <v>1</v>
@@ -3563,28 +3382,25 @@
       <c r="J59" t="b">
         <v>1</v>
       </c>
-      <c r="K59" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>172</v>
+        <v>142</v>
       </c>
       <c r="B60" t="s">
-        <v>173</v>
+        <v>11</v>
       </c>
       <c r="C60" t="s">
-        <v>75</v>
+        <v>11</v>
       </c>
       <c r="D60">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="E60" t="s">
-        <v>32</v>
-      </c>
-      <c r="F60" t="s">
-        <v>174</v>
+        <v>27</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>143</v>
       </c>
       <c r="G60" t="b">
         <v>1</v>
@@ -3598,28 +3414,25 @@
       <c r="J60" t="b">
         <v>1</v>
       </c>
-      <c r="K60" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>175</v>
+        <v>144</v>
       </c>
       <c r="B61" t="s">
-        <v>176</v>
+        <v>11</v>
       </c>
       <c r="C61" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="D61">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="E61" t="s">
-        <v>32</v>
-      </c>
-      <c r="F61" t="s">
-        <v>177</v>
+        <v>27</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>195</v>
       </c>
       <c r="G61" t="b">
         <v>1</v>
@@ -3633,28 +3446,25 @@
       <c r="J61" t="b">
         <v>1</v>
       </c>
-      <c r="K61" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>178</v>
+        <v>114</v>
       </c>
       <c r="B62" t="s">
-        <v>179</v>
+        <v>83</v>
       </c>
       <c r="C62" t="s">
-        <v>75</v>
+        <v>18</v>
       </c>
       <c r="D62">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="E62" t="s">
-        <v>13</v>
-      </c>
-      <c r="F62" t="s">
-        <v>180</v>
+        <v>27</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>162</v>
       </c>
       <c r="G62" t="b">
         <v>1</v>
@@ -3668,28 +3478,25 @@
       <c r="J62" t="b">
         <v>1</v>
       </c>
-      <c r="K62" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>181</v>
+        <v>145</v>
       </c>
       <c r="B63" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C63" t="s">
-        <v>64</v>
+        <v>96</v>
       </c>
       <c r="D63">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="E63" t="s">
-        <v>32</v>
-      </c>
-      <c r="F63" t="s">
-        <v>182</v>
+        <v>27</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>147</v>
       </c>
       <c r="G63" t="b">
         <v>1</v>
@@ -3703,28 +3510,25 @@
       <c r="J63" t="b">
         <v>1</v>
       </c>
-      <c r="K63" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>183</v>
+        <v>148</v>
       </c>
       <c r="B64" t="s">
-        <v>12</v>
+        <v>93</v>
       </c>
       <c r="C64" t="s">
-        <v>12</v>
+        <v>47</v>
       </c>
       <c r="D64">
         <v>2022</v>
       </c>
       <c r="E64" t="s">
-        <v>32</v>
-      </c>
-      <c r="F64" t="s">
-        <v>102</v>
+        <v>27</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>149</v>
       </c>
       <c r="G64" t="b">
         <v>1</v>
@@ -3738,28 +3542,25 @@
       <c r="J64" t="b">
         <v>1</v>
       </c>
-      <c r="K64" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>184</v>
+        <v>150</v>
       </c>
       <c r="B65" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C65" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D65">
         <v>2022</v>
       </c>
       <c r="E65" t="s">
-        <v>32</v>
-      </c>
-      <c r="F65" t="s">
-        <v>185</v>
+        <v>27</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>151</v>
       </c>
       <c r="G65" t="b">
         <v>1</v>
@@ -3773,203 +3574,185 @@
       <c r="J65" t="b">
         <v>1</v>
       </c>
-      <c r="K65" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
+        <v>152</v>
+      </c>
+      <c r="B66" t="s">
+        <v>83</v>
+      </c>
+      <c r="C66" t="s">
+        <v>18</v>
+      </c>
+      <c r="D66">
+        <v>2023</v>
+      </c>
+      <c r="E66" t="s">
+        <v>27</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="G66" t="b">
+        <v>1</v>
+      </c>
+      <c r="H66" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I66" t="b">
+        <v>0</v>
+      </c>
+      <c r="J66" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>153</v>
+      </c>
+      <c r="B67" t="s">
+        <v>43</v>
+      </c>
+      <c r="C67" t="s">
+        <v>33</v>
+      </c>
+      <c r="D67">
+        <v>2023</v>
+      </c>
+      <c r="E67" t="s">
+        <v>12</v>
+      </c>
+      <c r="F67" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="B66" t="s">
+      <c r="G67" t="b">
+        <v>1</v>
+      </c>
+      <c r="H67" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I67" t="b">
+        <v>0</v>
+      </c>
+      <c r="J67" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>154</v>
+      </c>
+      <c r="B68" t="s">
+        <v>11</v>
+      </c>
+      <c r="C68" t="s">
+        <v>11</v>
+      </c>
+      <c r="D68">
+        <v>2023</v>
+      </c>
+      <c r="E68" t="s">
+        <v>27</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="G68" t="b">
+        <v>1</v>
+      </c>
+      <c r="H68" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I68" t="b">
+        <v>0</v>
+      </c>
+      <c r="J68" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>156</v>
+      </c>
+      <c r="B69" t="s">
+        <v>11</v>
+      </c>
+      <c r="C69" t="s">
+        <v>11</v>
+      </c>
+      <c r="D69">
+        <v>2024</v>
+      </c>
+      <c r="E69" t="s">
+        <v>27</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="G69" t="b">
+        <v>1</v>
+      </c>
+      <c r="H69" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I69" t="b">
+        <v>0</v>
+      </c>
+      <c r="J69" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>157</v>
+      </c>
+      <c r="B70" t="s">
+        <v>83</v>
+      </c>
+      <c r="C70" t="s">
+        <v>18</v>
+      </c>
+      <c r="D70">
+        <v>2024</v>
+      </c>
+      <c r="E70" t="s">
         <v>12</v>
       </c>
-      <c r="C66" t="s">
+      <c r="F70" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G70" t="b">
+        <v>1</v>
+      </c>
+      <c r="H70" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I70" t="b">
+        <v>0</v>
+      </c>
+      <c r="J70" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>158</v>
+      </c>
+      <c r="B71" t="s">
+        <v>159</v>
+      </c>
+      <c r="C71" t="s">
+        <v>33</v>
+      </c>
+      <c r="D71">
+        <v>2025</v>
+      </c>
+      <c r="E71" t="s">
         <v>12</v>
       </c>
-      <c r="D66">
-        <v>2022</v>
-      </c>
-      <c r="E66" t="s">
-        <v>32</v>
-      </c>
-      <c r="F66" t="s">
-        <v>187</v>
-      </c>
-      <c r="G66" t="b">
-        <v>1</v>
-      </c>
-      <c r="H66" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I66" t="b">
-        <v>0</v>
-      </c>
-      <c r="J66" t="b">
-        <v>1</v>
-      </c>
-      <c r="K66" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A67" t="s">
-        <v>188</v>
-      </c>
-      <c r="B67" t="s">
-        <v>99</v>
-      </c>
-      <c r="C67" t="s">
-        <v>20</v>
-      </c>
-      <c r="D67">
-        <v>2022</v>
-      </c>
-      <c r="E67" t="s">
-        <v>32</v>
-      </c>
-      <c r="F67" t="s">
-        <v>174</v>
-      </c>
-      <c r="G67" t="b">
-        <v>1</v>
-      </c>
-      <c r="H67" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I67" t="b">
-        <v>0</v>
-      </c>
-      <c r="J67" t="b">
-        <v>1</v>
-      </c>
-      <c r="K67" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A68" t="s">
-        <v>189</v>
-      </c>
-      <c r="B68" t="s">
-        <v>190</v>
-      </c>
-      <c r="C68" t="s">
-        <v>120</v>
-      </c>
-      <c r="D68">
-        <v>2022</v>
-      </c>
-      <c r="E68" t="s">
-        <v>32</v>
-      </c>
-      <c r="F68" t="s">
-        <v>191</v>
-      </c>
-      <c r="G68" t="b">
-        <v>1</v>
-      </c>
-      <c r="H68" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I68" t="b">
-        <v>0</v>
-      </c>
-      <c r="J68" t="b">
-        <v>1</v>
-      </c>
-      <c r="K68" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
-        <v>192</v>
-      </c>
-      <c r="B69" t="s">
-        <v>115</v>
-      </c>
-      <c r="C69" t="s">
-        <v>56</v>
-      </c>
-      <c r="D69">
-        <v>2022</v>
-      </c>
-      <c r="E69" t="s">
-        <v>32</v>
-      </c>
-      <c r="F69" t="s">
-        <v>193</v>
-      </c>
-      <c r="G69" t="b">
-        <v>1</v>
-      </c>
-      <c r="H69" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I69" t="b">
-        <v>0</v>
-      </c>
-      <c r="J69" t="b">
-        <v>1</v>
-      </c>
-      <c r="K69" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
-        <v>194</v>
-      </c>
-      <c r="B70" t="s">
-        <v>12</v>
-      </c>
-      <c r="C70" t="s">
-        <v>12</v>
-      </c>
-      <c r="D70">
-        <v>2022</v>
-      </c>
-      <c r="E70" t="s">
-        <v>32</v>
-      </c>
-      <c r="F70" t="s">
-        <v>195</v>
-      </c>
-      <c r="G70" t="b">
-        <v>1</v>
-      </c>
-      <c r="H70" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I70" t="b">
-        <v>0</v>
-      </c>
-      <c r="J70" t="b">
-        <v>1</v>
-      </c>
-      <c r="K70" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A71" t="s">
-        <v>196</v>
-      </c>
-      <c r="B71" t="s">
-        <v>99</v>
-      </c>
-      <c r="C71" t="s">
-        <v>20</v>
-      </c>
-      <c r="D71">
-        <v>2023</v>
-      </c>
-      <c r="E71" t="s">
-        <v>32</v>
-      </c>
-      <c r="F71" t="s">
-        <v>110</v>
+      <c r="F71" s="2" t="s">
+        <v>198</v>
       </c>
       <c r="G71" t="b">
         <v>1</v>
@@ -3983,186 +3766,80 @@
       <c r="J71" t="b">
         <v>1</v>
       </c>
-      <c r="K71" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A72" t="s">
-        <v>197</v>
-      </c>
-      <c r="B72" t="s">
-        <v>52</v>
-      </c>
-      <c r="C72" t="s">
-        <v>39</v>
-      </c>
-      <c r="D72">
-        <v>2023</v>
-      </c>
-      <c r="E72" t="s">
-        <v>13</v>
-      </c>
-      <c r="F72" t="s">
-        <v>198</v>
-      </c>
-      <c r="G72" t="b">
-        <v>1</v>
-      </c>
-      <c r="H72" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I72" t="b">
-        <v>0</v>
-      </c>
-      <c r="J72" t="b">
-        <v>1</v>
-      </c>
-      <c r="K72" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
-        <v>199</v>
-      </c>
-      <c r="B73" t="s">
-        <v>12</v>
-      </c>
-      <c r="C73" t="s">
-        <v>12</v>
-      </c>
-      <c r="D73">
-        <v>2023</v>
-      </c>
-      <c r="E73" t="s">
-        <v>32</v>
-      </c>
-      <c r="F73" t="s">
-        <v>200</v>
-      </c>
-      <c r="G73" t="b">
-        <v>1</v>
-      </c>
-      <c r="H73" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I73" t="b">
-        <v>0</v>
-      </c>
-      <c r="J73" t="b">
-        <v>1</v>
-      </c>
-      <c r="K73" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
-        <v>201</v>
-      </c>
-      <c r="B74" t="s">
-        <v>12</v>
-      </c>
-      <c r="C74" t="s">
-        <v>12</v>
-      </c>
-      <c r="D74">
-        <v>2024</v>
-      </c>
-      <c r="E74" t="s">
-        <v>32</v>
-      </c>
-      <c r="F74" t="s">
-        <v>195</v>
-      </c>
-      <c r="G74" t="b">
-        <v>1</v>
-      </c>
-      <c r="H74" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I74" t="b">
-        <v>0</v>
-      </c>
-      <c r="J74" t="b">
-        <v>1</v>
-      </c>
-      <c r="K74" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A75" t="s">
-        <v>202</v>
-      </c>
-      <c r="B75" t="s">
-        <v>99</v>
-      </c>
-      <c r="C75" t="s">
-        <v>20</v>
-      </c>
-      <c r="D75">
-        <v>2024</v>
-      </c>
-      <c r="E75" t="s">
-        <v>13</v>
-      </c>
-      <c r="F75" t="s">
-        <v>110</v>
-      </c>
-      <c r="G75" t="b">
-        <v>1</v>
-      </c>
-      <c r="H75" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I75" t="b">
-        <v>0</v>
-      </c>
-      <c r="J75" t="b">
-        <v>1</v>
-      </c>
-      <c r="K75" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
-        <v>203</v>
-      </c>
-      <c r="B76" t="s">
-        <v>204</v>
-      </c>
-      <c r="C76" t="s">
-        <v>39</v>
-      </c>
-      <c r="D76">
-        <v>2025</v>
-      </c>
-      <c r="E76" t="s">
-        <v>13</v>
-      </c>
-      <c r="F76" t="s">
-        <v>205</v>
-      </c>
-      <c r="G76" t="b">
-        <v>1</v>
-      </c>
-      <c r="H76" s="1">
-        <v>46138</v>
-      </c>
-      <c r="I76" t="b">
-        <v>0</v>
-      </c>
-      <c r="J76" t="b">
-        <v>1</v>
-      </c>
-      <c r="K76" t="s">
-        <v>165</v>
-      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F62" r:id="rId1" xr:uid="{673AF8FD-8728-4E58-BA67-A5E7BF1618FF}"/>
+    <hyperlink ref="F59" r:id="rId2" xr:uid="{9512233A-183C-4A57-9F44-6963665C8620}"/>
+    <hyperlink ref="F7" r:id="rId3" xr:uid="{47F19EE5-A9C9-4602-9C2C-C64F497AE76F}"/>
+    <hyperlink ref="F2" r:id="rId4" xr:uid="{091C4D4B-0E48-4F65-8095-EF79AA772967}"/>
+    <hyperlink ref="F4" r:id="rId5" xr:uid="{F207ABC6-5B0C-4CE6-BCA6-591F1DB50A07}"/>
+    <hyperlink ref="F5" r:id="rId6" xr:uid="{535B15C8-A1C1-4FA7-97F9-9161930622D6}"/>
+    <hyperlink ref="F9" r:id="rId7" xr:uid="{1EB00C34-B020-4DF5-8D59-9ACC37C73C3A}"/>
+    <hyperlink ref="F10" r:id="rId8" xr:uid="{650F1F8A-C228-4F9C-A830-4605239D476E}"/>
+    <hyperlink ref="F11" r:id="rId9" xr:uid="{FDB6D38B-5EFF-4DC8-9209-A04E6C8E2794}"/>
+    <hyperlink ref="F12" r:id="rId10" xr:uid="{C051C68C-CA18-4737-840A-3FA99A301060}"/>
+    <hyperlink ref="F13" r:id="rId11" xr:uid="{6FB709DF-F5A0-4B32-AD44-C1B611C6D0F3}"/>
+    <hyperlink ref="F14" r:id="rId12" xr:uid="{42231A39-B051-45D1-9E03-B052C31F536A}"/>
+    <hyperlink ref="F16" r:id="rId13" xr:uid="{9A63680B-594B-4AAA-9139-7190BAE8FD1B}"/>
+    <hyperlink ref="F17" r:id="rId14" xr:uid="{5FFE15F8-8480-4E9E-AF96-AE7289D14F9D}"/>
+    <hyperlink ref="F18" r:id="rId15" xr:uid="{151D357B-734E-4C4F-9B19-0DB730382C37}"/>
+    <hyperlink ref="F19" r:id="rId16" xr:uid="{267F4FC9-27F9-4165-86A1-74D2B60596C2}"/>
+    <hyperlink ref="F20" r:id="rId17" xr:uid="{356A054B-EA9D-46DA-8FB4-333E9D4979D0}"/>
+    <hyperlink ref="F21" r:id="rId18" xr:uid="{C813CF9B-A00C-433D-AD6A-8EDA9E030EF6}"/>
+    <hyperlink ref="F22" r:id="rId19" xr:uid="{B21CC331-2178-4974-AA60-8FFC7B63559B}"/>
+    <hyperlink ref="F23" r:id="rId20" xr:uid="{F8B3F542-B90B-4A0E-A7AB-E207ECC39064}"/>
+    <hyperlink ref="F24" r:id="rId21" xr:uid="{91C1683A-BE37-4D01-986F-A84456DD253A}"/>
+    <hyperlink ref="F25" r:id="rId22" xr:uid="{EE03F542-A349-4FAA-AD7B-BD5B0DD253BF}"/>
+    <hyperlink ref="F26" r:id="rId23" xr:uid="{1C19A78F-33CF-4C48-B326-776463419BC6}"/>
+    <hyperlink ref="F27" r:id="rId24" xr:uid="{5EEAC673-FB35-4512-AB0E-BE2E62F5A1E1}"/>
+    <hyperlink ref="F28" r:id="rId25" xr:uid="{BD89DB79-06AD-495A-B967-8010024E9DB8}"/>
+    <hyperlink ref="F29" r:id="rId26" xr:uid="{5C0DF011-D308-417D-B017-A3DF7C7658B5}"/>
+    <hyperlink ref="F30" r:id="rId27" xr:uid="{41B05A55-4116-4F72-9C90-23247E4CE981}"/>
+    <hyperlink ref="F31" r:id="rId28" xr:uid="{EA234A99-93F9-4E94-8F89-8C6B0E06D975}"/>
+    <hyperlink ref="F32" r:id="rId29" xr:uid="{71270214-D984-4437-8867-13F911B87402}"/>
+    <hyperlink ref="F33" r:id="rId30" xr:uid="{8BAC703C-FEFC-42EC-9A29-6C8274C4B331}"/>
+    <hyperlink ref="F34" r:id="rId31" xr:uid="{D8A6AA8E-E204-4A72-858B-60FE9165AE8F}"/>
+    <hyperlink ref="F35" r:id="rId32" xr:uid="{051842CC-67B5-42FD-93CA-1EB2F5D19043}"/>
+    <hyperlink ref="F36" r:id="rId33" xr:uid="{3A0DB7BE-7DAA-4F9A-97C9-1901F1B4521A}"/>
+    <hyperlink ref="F37" r:id="rId34" xr:uid="{FC9B24A8-225D-413A-AF95-17D2B01E9ADD}"/>
+    <hyperlink ref="F38" r:id="rId35" xr:uid="{8E1E9709-5D5D-4964-ABF0-F8E9F52A5BDA}"/>
+    <hyperlink ref="F39" r:id="rId36" xr:uid="{FFE62EC2-BBE6-4A18-B79C-EA860123F9F7}"/>
+    <hyperlink ref="F40" r:id="rId37" xr:uid="{12568B6A-2226-4D70-AAA2-3AC7F7D2D4E3}"/>
+    <hyperlink ref="F41" r:id="rId38" xr:uid="{8F195DF5-544E-4474-A5DA-87EC29219FD4}"/>
+    <hyperlink ref="F42" r:id="rId39" xr:uid="{196395EB-615C-4FCB-AA52-2F836A90CCBE}"/>
+    <hyperlink ref="F43" r:id="rId40" xr:uid="{A89E6CFF-FEA5-4F53-AFEE-5512170A08B2}"/>
+    <hyperlink ref="F44" r:id="rId41" xr:uid="{07701988-D506-4D40-AC4E-45CE2C43B289}"/>
+    <hyperlink ref="F45" r:id="rId42" xr:uid="{86B95A67-CD7B-40E1-BF35-316D9294C9C3}"/>
+    <hyperlink ref="F46" r:id="rId43" xr:uid="{9AAC29C9-4CA4-460C-BC08-7D1E71833DE0}"/>
+    <hyperlink ref="F47" r:id="rId44" xr:uid="{13764CB2-7613-4B0C-8940-D649C845ADC6}"/>
+    <hyperlink ref="F48" r:id="rId45" xr:uid="{3BC330F1-DF21-4EF6-827E-E447B4205F0E}"/>
+    <hyperlink ref="F49" r:id="rId46" xr:uid="{BA2999EB-AB8A-491D-9C19-B53C47E7E9CB}"/>
+    <hyperlink ref="F50" r:id="rId47" xr:uid="{967177E6-C603-4CB8-ABF2-ABD2E9972550}"/>
+    <hyperlink ref="F51" r:id="rId48" xr:uid="{8518A56A-AB79-473E-A6CA-83B5EF1C35D3}"/>
+    <hyperlink ref="F52" r:id="rId49" xr:uid="{0DC81FDC-9BB8-451E-A5EB-F9D8B8D1E421}"/>
+    <hyperlink ref="F53" r:id="rId50" xr:uid="{41E1BEA3-E4A4-4443-8A00-0E6A7F316FF6}"/>
+    <hyperlink ref="F54" r:id="rId51" xr:uid="{513DF9A4-6FAE-4536-9CCE-6F44A5A86FC2}"/>
+    <hyperlink ref="F55" r:id="rId52" xr:uid="{E31AF7E0-C3B7-4148-94ED-FE17960BB243}"/>
+    <hyperlink ref="F56" r:id="rId53" xr:uid="{0CB36533-994E-4331-BD8C-34DB07EE4325}"/>
+    <hyperlink ref="F57" r:id="rId54" xr:uid="{76AAE522-9542-40FF-9700-7F877B9716F2}"/>
+    <hyperlink ref="F58" r:id="rId55" xr:uid="{0AE920B0-1A8D-44C5-B3C5-F24C1BBDFF80}"/>
+    <hyperlink ref="F60" r:id="rId56" xr:uid="{C90ECE11-BE7D-492C-9376-23DC23BA593A}"/>
+    <hyperlink ref="F61" r:id="rId57" xr:uid="{202BDFB4-D2B1-4BAC-93F1-1CE7F7C74B47}"/>
+    <hyperlink ref="F63" r:id="rId58" xr:uid="{87FEE190-912E-49AE-8B1B-859FDF1AB3C9}"/>
+    <hyperlink ref="F64" r:id="rId59" xr:uid="{1C20B4E8-1CBB-4C57-B2E6-A7C4381B073E}"/>
+    <hyperlink ref="F65" r:id="rId60" xr:uid="{00D54F8A-16C2-491A-A855-DFCF540A5E26}"/>
+    <hyperlink ref="F66" r:id="rId61" display="https://www.depotclimbing.co.uk/manchester/?_gl=1%2Aq9klp8%2A_up%2AMQ..%2A_ga%2ANTg0MzYxNDYzLjE3NzgyMjYzMjk.%2A_ga_7TXZCZ3B9X%2AczE3NzgyMjYzMjgkbzEkZzAkdDE3NzgyMjYzMjgkajYwJGwwJGgw%2A_ga_XKDQRJ4PB4%2AczE3NzgyMjYzMjgkbzEkZzAkdDE3NzgyMjYzMjgkajYwJGwwJGg3NTkzODk3MjM." xr:uid="{34455584-87B5-4E9C-A4FF-4A46FFD8E460}"/>
+    <hyperlink ref="F67" r:id="rId62" xr:uid="{FF38188C-B00D-40AA-BE66-22ABE72C7F4A}"/>
+    <hyperlink ref="F68" r:id="rId63" xr:uid="{7F316393-F68F-4C80-84B8-282E3962C86A}"/>
+    <hyperlink ref="F69" r:id="rId64" xr:uid="{B4F2D5C5-40F1-45BF-9867-CA0380541529}"/>
+    <hyperlink ref="F70" r:id="rId65" xr:uid="{7CF45127-3F0D-4ED5-BFF9-AE8E70D630B7}"/>
+    <hyperlink ref="F71" r:id="rId66" xr:uid="{D43183AF-A8B8-450B-A754-620A257D41DB}"/>
+    <hyperlink ref="F3" r:id="rId67" xr:uid="{83585F05-B679-4AA3-87DB-8C1408FA344E}"/>
+    <hyperlink ref="F6" r:id="rId68" xr:uid="{AB23C56B-52B7-4506-8953-40076D58B2F9}"/>
+    <hyperlink ref="F8" r:id="rId69" xr:uid="{64C8C531-8AAF-46EC-A6C7-A0B184331AD1}"/>
+    <hyperlink ref="F15" r:id="rId70" xr:uid="{4CA1CEDF-571B-4048-B082-79E7A2D8B8BC}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>